<commit_message>
Encore plus de données + des magnifiques graphiques
</commit_message>
<xml_diff>
--- a/excel/backup.xlsx
+++ b/excel/backup.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="29">
   <si>
     <t xml:space="preserve">nom</t>
   </si>
@@ -397,10 +397,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O39"/>
+  <dimension ref="A1:O68"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="0" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2231,6 +2231,1369 @@
       </c>
       <c r="O39" s="0" t="n">
         <v>0.00191577208918249</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C40" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D40" s="0" t="n">
+        <v>1041</v>
+      </c>
+      <c r="E40" s="0" t="n">
+        <v>462</v>
+      </c>
+      <c r="F40" s="0" t="n">
+        <v>480942</v>
+      </c>
+      <c r="G40" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H40" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="I40" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="J40" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="K40" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" s="0" t="n">
+        <v>12.0404679775238</v>
+      </c>
+      <c r="M40" s="0" t="n">
+        <v>10.0250902175903</v>
+      </c>
+      <c r="N40" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C41" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D41" s="0" t="n">
+        <v>1041</v>
+      </c>
+      <c r="E41" s="0" t="n">
+        <v>462</v>
+      </c>
+      <c r="F41" s="0" t="n">
+        <v>480942</v>
+      </c>
+      <c r="G41" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H41" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="I41" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="J41" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="K41" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="L41" s="0" t="n">
+        <v>17.4147531986237</v>
+      </c>
+      <c r="M41" s="0" t="n">
+        <v>23.1594908237457</v>
+      </c>
+      <c r="N41" s="0" t="n">
+        <v>0.000804670833489277</v>
+      </c>
+      <c r="O41" s="0" t="n">
+        <v>0.000773482041493569</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C42" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D42" s="0" t="n">
+        <v>1041</v>
+      </c>
+      <c r="E42" s="0" t="n">
+        <v>462</v>
+      </c>
+      <c r="F42" s="0" t="n">
+        <v>480942</v>
+      </c>
+      <c r="G42" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H42" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="I42" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="J42" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="K42" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="L42" s="0" t="n">
+        <v>18.0342693328857</v>
+      </c>
+      <c r="M42" s="0" t="n">
+        <v>25.4128968715668</v>
+      </c>
+      <c r="N42" s="0" t="n">
+        <v>0.0135941548045294</v>
+      </c>
+      <c r="O42" s="0" t="n">
+        <v>0.0125087848430788</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C43" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D43" s="0" t="n">
+        <v>1041</v>
+      </c>
+      <c r="E43" s="0" t="n">
+        <v>462</v>
+      </c>
+      <c r="F43" s="0" t="n">
+        <v>480942</v>
+      </c>
+      <c r="G43" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H43" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="I43" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="J43" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="K43" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="L43" s="0" t="n">
+        <v>19.3115365505219</v>
+      </c>
+      <c r="M43" s="0" t="n">
+        <v>21.4742527008057</v>
+      </c>
+      <c r="N43" s="0" t="n">
+        <v>0.0751275621592625</v>
+      </c>
+      <c r="O43" s="0" t="n">
+        <v>0.0678668113826615</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C44" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D44" s="0" t="n">
+        <v>1041</v>
+      </c>
+      <c r="E44" s="0" t="n">
+        <v>462</v>
+      </c>
+      <c r="F44" s="0" t="n">
+        <v>480942</v>
+      </c>
+      <c r="G44" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H44" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="I44" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="J44" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="K44" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="L44" s="0" t="n">
+        <v>20.1335628032684</v>
+      </c>
+      <c r="M44" s="0" t="n">
+        <v>20.3449144363403</v>
+      </c>
+      <c r="N44" s="0" t="n">
+        <v>0.122072931871203</v>
+      </c>
+      <c r="O44" s="0" t="n">
+        <v>0.107220829122846</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C45" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D45" s="0" t="n">
+        <v>1041</v>
+      </c>
+      <c r="E45" s="0" t="n">
+        <v>462</v>
+      </c>
+      <c r="F45" s="0" t="n">
+        <v>480942</v>
+      </c>
+      <c r="G45" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H45" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="I45" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="J45" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="K45" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="L45" s="0" t="n">
+        <v>20.5345215797424</v>
+      </c>
+      <c r="M45" s="0" t="n">
+        <v>20.1428418159485</v>
+      </c>
+      <c r="N45" s="0" t="n">
+        <v>0.152926964166157</v>
+      </c>
+      <c r="O45" s="0" t="n">
+        <v>0.13067064219802</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C46" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D46" s="0" t="n">
+        <v>1041</v>
+      </c>
+      <c r="E46" s="0" t="n">
+        <v>462</v>
+      </c>
+      <c r="F46" s="0" t="n">
+        <v>480942</v>
+      </c>
+      <c r="G46" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H46" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="I46" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="J46" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="K46" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="L46" s="0" t="n">
+        <v>20.4464023113251</v>
+      </c>
+      <c r="M46" s="0" t="n">
+        <v>20.3424112796783</v>
+      </c>
+      <c r="N46" s="0" t="n">
+        <v>0.182537603286883</v>
+      </c>
+      <c r="O46" s="0" t="n">
+        <v>0.150853949124843</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C47" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D47" s="0" t="n">
+        <v>1041</v>
+      </c>
+      <c r="E47" s="0" t="n">
+        <v>462</v>
+      </c>
+      <c r="F47" s="0" t="n">
+        <v>480942</v>
+      </c>
+      <c r="G47" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H47" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="I47" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="J47" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="K47" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="L47" s="0" t="n">
+        <v>20.6530771255493</v>
+      </c>
+      <c r="M47" s="0" t="n">
+        <v>21.2032210826874</v>
+      </c>
+      <c r="N47" s="0" t="n">
+        <v>0.212848950601112</v>
+      </c>
+      <c r="O47" s="0" t="n">
+        <v>0.170839727035692</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C48" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D48" s="0" t="n">
+        <v>1041</v>
+      </c>
+      <c r="E48" s="0" t="n">
+        <v>462</v>
+      </c>
+      <c r="F48" s="0" t="n">
+        <v>480942</v>
+      </c>
+      <c r="G48" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H48" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="I48" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="J48" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="K48" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="L48" s="0" t="n">
+        <v>21.1984617710114</v>
+      </c>
+      <c r="M48" s="0" t="n">
+        <v>23.7816650867462</v>
+      </c>
+      <c r="N48" s="0" t="n">
+        <v>0.242844251489785</v>
+      </c>
+      <c r="O48" s="0" t="n">
+        <v>0.187837618673354</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="1" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C49" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D49" s="0" t="n">
+        <v>1041</v>
+      </c>
+      <c r="E49" s="0" t="n">
+        <v>462</v>
+      </c>
+      <c r="F49" s="0" t="n">
+        <v>480942</v>
+      </c>
+      <c r="G49" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H49" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="I49" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="J49" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="K49" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="L49" s="0" t="n">
+        <v>21.2840340137482</v>
+      </c>
+      <c r="M49" s="0" t="n">
+        <v>23.7993264198303</v>
+      </c>
+      <c r="N49" s="0" t="n">
+        <v>0.27209102137056</v>
+      </c>
+      <c r="O49" s="0" t="n">
+        <v>0.204284508319091</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C50" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D50" s="0" t="n">
+        <v>1041</v>
+      </c>
+      <c r="E50" s="0" t="n">
+        <v>462</v>
+      </c>
+      <c r="F50" s="0" t="n">
+        <v>480942</v>
+      </c>
+      <c r="G50" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H50" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="I50" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="J50" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="K50" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="L50" s="0" t="n">
+        <v>21.4926390647888</v>
+      </c>
+      <c r="M50" s="0" t="n">
+        <v>21.317681312561</v>
+      </c>
+      <c r="N50" s="0" t="n">
+        <v>0.301840970428867</v>
+      </c>
+      <c r="O50" s="0" t="n">
+        <v>0.219845636272149</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="1" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C51" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="D51" s="0" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E51" s="0" t="n">
+        <v>157</v>
+      </c>
+      <c r="F51" s="0" t="n">
+        <v>164850</v>
+      </c>
+      <c r="G51" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="H51" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="I51" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="J51" s="0" t="n">
+        <v>87</v>
+      </c>
+      <c r="K51" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L51" s="0" t="n">
+        <v>16.3122532367706</v>
+      </c>
+      <c r="M51" s="0" t="n">
+        <v>29.3742055892944</v>
+      </c>
+      <c r="N51" s="0" t="n">
+        <v>0.0106339096148013</v>
+      </c>
+      <c r="O51" s="0" t="n">
+        <v>0.00951774340309372</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C52" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="D52" s="0" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E52" s="0" t="n">
+        <v>157</v>
+      </c>
+      <c r="F52" s="0" t="n">
+        <v>164850</v>
+      </c>
+      <c r="G52" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="H52" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="I52" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="J52" s="0" t="n">
+        <v>77</v>
+      </c>
+      <c r="K52" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L52" s="0" t="n">
+        <v>12.8161981105804</v>
+      </c>
+      <c r="M52" s="0" t="n">
+        <v>20.9182598590851</v>
+      </c>
+      <c r="N52" s="0" t="n">
+        <v>0.014540491355778</v>
+      </c>
+      <c r="O52" s="0" t="n">
+        <v>0.0131877464361541</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C53" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="D53" s="0" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E53" s="0" t="n">
+        <v>157</v>
+      </c>
+      <c r="F53" s="0" t="n">
+        <v>164850</v>
+      </c>
+      <c r="G53" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="H53" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="I53" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="J53" s="0" t="n">
+        <v>67</v>
+      </c>
+      <c r="K53" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L53" s="0" t="n">
+        <v>11.4995164871216</v>
+      </c>
+      <c r="M53" s="0" t="n">
+        <v>17.5519821643829</v>
+      </c>
+      <c r="N53" s="0" t="n">
+        <v>0.0227540188049742</v>
+      </c>
+      <c r="O53" s="0" t="n">
+        <v>0.020060661207158</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C54" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="D54" s="0" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E54" s="0" t="n">
+        <v>157</v>
+      </c>
+      <c r="F54" s="0" t="n">
+        <v>164850</v>
+      </c>
+      <c r="G54" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H54" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="I54" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="J54" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="K54" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L54" s="0" t="n">
+        <v>9.88741374015808</v>
+      </c>
+      <c r="M54" s="0" t="n">
+        <v>14.4777653217316</v>
+      </c>
+      <c r="N54" s="0" t="n">
+        <v>0.0335395814376706</v>
+      </c>
+      <c r="O54" s="0" t="n">
+        <v>0.0293964209887777</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="1" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C55" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="D55" s="0" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E55" s="0" t="n">
+        <v>157</v>
+      </c>
+      <c r="F55" s="0" t="n">
+        <v>164850</v>
+      </c>
+      <c r="G55" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="H55" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="I55" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="J55" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="K55" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L55" s="0" t="n">
+        <v>9.76782202720642</v>
+      </c>
+      <c r="M55" s="0" t="n">
+        <v>13.7494201660156</v>
+      </c>
+      <c r="N55" s="0" t="n">
+        <v>0.0531938125568699</v>
+      </c>
+      <c r="O55" s="0" t="n">
+        <v>0.0470063694267516</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="1" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C56" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="D56" s="0" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E56" s="0" t="n">
+        <v>157</v>
+      </c>
+      <c r="F56" s="0" t="n">
+        <v>164850</v>
+      </c>
+      <c r="G56" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="H56" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="I56" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="J56" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="K56" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L56" s="0" t="n">
+        <v>8.05767846107483</v>
+      </c>
+      <c r="M56" s="0" t="n">
+        <v>9.524653673172</v>
+      </c>
+      <c r="N56" s="0" t="n">
+        <v>0.0760206248104337</v>
+      </c>
+      <c r="O56" s="0" t="n">
+        <v>0.0679526842584168</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="1" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C57" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D57" s="0" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E57" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="F57" s="0" t="n">
+        <v>608400</v>
+      </c>
+      <c r="G57" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H57" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="I57" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="K57" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L57" s="0" t="n">
+        <v>30.8922982215881</v>
+      </c>
+      <c r="M57" s="0" t="n">
+        <v>29.5011813640595</v>
+      </c>
+      <c r="N57" s="0" t="n">
+        <v>0.0996400394477318</v>
+      </c>
+      <c r="O57" s="0" t="n">
+        <v>0.0894773175542406</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="1" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C58" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D58" s="0" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E58" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="F58" s="0" t="n">
+        <v>608400</v>
+      </c>
+      <c r="G58" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H58" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="I58" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="J58" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="K58" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L58" s="0" t="n">
+        <v>35.1273875236511</v>
+      </c>
+      <c r="M58" s="0" t="n">
+        <v>34.3286054134369</v>
+      </c>
+      <c r="N58" s="0" t="n">
+        <v>0.102618343195266</v>
+      </c>
+      <c r="O58" s="0" t="n">
+        <v>0.092000328731098</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="1" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C59" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D59" s="0" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E59" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="F59" s="0" t="n">
+        <v>608400</v>
+      </c>
+      <c r="G59" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H59" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="I59" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="J59" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="K59" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L59" s="0" t="n">
+        <v>35.978688955307</v>
+      </c>
+      <c r="M59" s="0" t="n">
+        <v>38.2744550704956</v>
+      </c>
+      <c r="N59" s="0" t="n">
+        <v>0.0983053911900066</v>
+      </c>
+      <c r="O59" s="0" t="n">
+        <v>0.088198553583169</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="1" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C60" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D60" s="0" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E60" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="F60" s="0" t="n">
+        <v>608400</v>
+      </c>
+      <c r="G60" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H60" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="I60" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="J60" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="K60" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L60" s="0" t="n">
+        <v>38.5633368492127</v>
+      </c>
+      <c r="M60" s="0" t="n">
+        <v>42.0682859420776</v>
+      </c>
+      <c r="N60" s="0" t="n">
+        <v>0.0759253780407627</v>
+      </c>
+      <c r="O60" s="0" t="n">
+        <v>0.0670562130177515</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="1" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C61" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D61" s="0" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E61" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="F61" s="0" t="n">
+        <v>608400</v>
+      </c>
+      <c r="G61" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H61" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="I61" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="J61" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="K61" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L61" s="0" t="n">
+        <v>45.6055269241333</v>
+      </c>
+      <c r="M61" s="0" t="n">
+        <v>59.2971668243408</v>
+      </c>
+      <c r="N61" s="0" t="n">
+        <v>0.0398487836949375</v>
+      </c>
+      <c r="O61" s="0" t="n">
+        <v>0.0351019066403682</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C62" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D62" s="0" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E62" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="F62" s="0" t="n">
+        <v>608400</v>
+      </c>
+      <c r="G62" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H62" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="I62" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="J62" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="K62" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L62" s="0" t="n">
+        <v>45.7633092403412</v>
+      </c>
+      <c r="M62" s="0" t="n">
+        <v>96.55042719841</v>
+      </c>
+      <c r="N62" s="0" t="n">
+        <v>0.0177087442472058</v>
+      </c>
+      <c r="O62" s="0" t="n">
+        <v>0.0156426692965155</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="1" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C63" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D63" s="0" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E63" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="F63" s="0" t="n">
+        <v>608400</v>
+      </c>
+      <c r="G63" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H63" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="I63" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="J63" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="K63" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L63" s="0" t="n">
+        <v>48.2481248378754</v>
+      </c>
+      <c r="M63" s="0" t="n">
+        <v>167.032883405685</v>
+      </c>
+      <c r="N63" s="0" t="n">
+        <v>0.0116058514135437</v>
+      </c>
+      <c r="O63" s="0" t="n">
+        <v>0.0104240631163708</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="1" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C64" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D64" s="0" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E64" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="F64" s="0" t="n">
+        <v>608400</v>
+      </c>
+      <c r="G64" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H64" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="I64" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="J64" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="K64" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L64" s="0" t="n">
+        <v>53.6992161273956</v>
+      </c>
+      <c r="M64" s="0" t="n">
+        <v>278.312934875488</v>
+      </c>
+      <c r="N64" s="0" t="n">
+        <v>0.00939677843523997</v>
+      </c>
+      <c r="O64" s="0" t="n">
+        <v>0.00851413543721236</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="1" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C65" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D65" s="0" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E65" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="F65" s="0" t="n">
+        <v>608400</v>
+      </c>
+      <c r="G65" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H65" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="I65" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="J65" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="K65" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L65" s="0" t="n">
+        <v>54.3164167404175</v>
+      </c>
+      <c r="M65" s="0" t="n">
+        <v>430.646780252457</v>
+      </c>
+      <c r="N65" s="0" t="n">
+        <v>0.00973865877712032</v>
+      </c>
+      <c r="O65" s="0" t="n">
+        <v>0.00880670611439842</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="B66" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C66" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D66" s="0" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E66" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="F66" s="0" t="n">
+        <v>608400</v>
+      </c>
+      <c r="G66" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H66" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="I66" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="J66" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="K66" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L66" s="0" t="n">
+        <v>57.6310431957245</v>
+      </c>
+      <c r="M66" s="0" t="n">
+        <v>623.742655038834</v>
+      </c>
+      <c r="N66" s="0" t="n">
+        <v>0.0102186061801446</v>
+      </c>
+      <c r="O66" s="0" t="n">
+        <v>0.00908941485864563</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C67" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D67" s="0" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E67" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="F67" s="0" t="n">
+        <v>608400</v>
+      </c>
+      <c r="G67" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H67" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="I67" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="J67" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="K67" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L67" s="0" t="n">
+        <v>64.0548136234283</v>
+      </c>
+      <c r="M67" s="0" t="n">
+        <v>907.425092935562</v>
+      </c>
+      <c r="N67" s="0" t="n">
+        <v>0.00987179487179487</v>
+      </c>
+      <c r="O67" s="0" t="n">
+        <v>0.00896942800788955</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="1" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C68" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D68" s="0" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E68" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="F68" s="0" t="n">
+        <v>608400</v>
+      </c>
+      <c r="G68" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="H68" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="I68" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="J68" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="K68" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="L68" s="0" t="n">
+        <v>63.5185508728027</v>
+      </c>
+      <c r="M68" s="0" t="n">
+        <v>1238.25290942192</v>
+      </c>
+      <c r="N68" s="0" t="n">
+        <v>0.00972550953320184</v>
+      </c>
+      <c r="O68" s="0" t="n">
+        <v>0.00872616699539777</v>
       </c>
     </row>
   </sheetData>

</xml_diff>